<commit_message>
W-1 and LEM-1: the drawing build re-recorded on all five models with a new project naming no surface family (owner 173 a)
No build reply reports a family switch. Opus 5.5 right on both columns
(1.2441; it widened the ground both ways and said so); Sonnet 5.5's reply
misstates the left extent it built (6 of 8 explanation, was 7); Kimi K3's
"tangent to the rock" slip gone (5 of 8, was 4); GLM-5V-Turbo drew the
foundation line along the ground surface and reported 1.856 (wrong model,
as before); gpt-6-astra right. Opus total $0.93; the other four $0.25-$1.30.
LEM-1's build re-solves to 1.2758 (published 1.276); its paragraph describes
only what the figure shows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_build_from_image_after.xlsx
+++ b/docs/tutorials/files/w1_build_from_image_after.xlsx
@@ -10615,7 +10615,7 @@
         <v>20.0</v>
       </c>
       <c r="D10" s="3">
-        <v>0.0</v>
+        <v>130.0</v>
       </c>
       <c r="E10" s="3">
         <v>0.0</v>
@@ -10657,17 +10657,13 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>90.0</v>
+        <v>130.0</v>
       </c>
       <c r="B11" s="3">
         <v>20.0</v>
       </c>
-      <c r="D11" s="3">
-        <v>90.0</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.0</v>
-      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="3"/>

</xml_diff>